<commit_message>
Implement exact format preservation and Pallet column generation with ExcelJS
</commit_message>
<xml_diff>
--- a/Sample/11. Total OB request - 20.05.2026.xlsx
+++ b/Sample/11. Total OB request - 20.05.2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\AI Learning\OBOUND\Tháng 5\Ngày 22.5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\AI Learning\Generate ASN\Sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1742" documentId="13_ncr:1_{7325AF9C-B8FE-4824-8512-7C76444D8D0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DED7B7FC-9AEB-428D-ACE4-DAA49A9B6A18}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334F1191-7F71-4308-9F3C-0EABB62928CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="746" activeTab="1" xr2:uid="{7E9943A3-A868-4900-9880-FF41B483368D}"/>
   </bookViews>
@@ -268,7 +268,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="127">
   <si>
     <t>Customer PO</t>
   </si>
@@ -664,6 +664,9 @@
   </si>
   <si>
     <t>PO5-0526_T4</t>
+  </si>
+  <si>
+    <t>Số lượng pallet</t>
   </si>
 </sst>
 </file>
@@ -1303,7 +1306,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="131">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1612,7 +1615,6 @@
     <xf numFmtId="43" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="16" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2175,10 +2177,10 @@
         <v>6.2</v>
       </c>
       <c r="P3" s="106"/>
-      <c r="Q3" s="128" t="s">
+      <c r="Q3" s="127" t="s">
         <v>81</v>
       </c>
-      <c r="R3" s="130"/>
+      <c r="R3" s="129"/>
       <c r="T3" s="77"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.35">
@@ -2228,8 +2230,8 @@
         <v>6.2</v>
       </c>
       <c r="P4" s="97"/>
-      <c r="Q4" s="129"/>
-      <c r="R4" s="131"/>
+      <c r="Q4" s="128"/>
+      <c r="R4" s="130"/>
       <c r="T4" s="77"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.35">
@@ -2279,8 +2281,8 @@
         <v>6.2</v>
       </c>
       <c r="P5" s="97"/>
-      <c r="Q5" s="129"/>
-      <c r="R5" s="131"/>
+      <c r="Q5" s="128"/>
+      <c r="R5" s="130"/>
       <c r="T5" s="77"/>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.35">
@@ -2330,8 +2332,8 @@
         <v>6.2</v>
       </c>
       <c r="P6" s="97"/>
-      <c r="Q6" s="129"/>
-      <c r="R6" s="131"/>
+      <c r="Q6" s="128"/>
+      <c r="R6" s="130"/>
       <c r="T6" s="77"/>
     </row>
     <row r="7" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2381,8 +2383,8 @@
         <v>6.15</v>
       </c>
       <c r="P7" s="97"/>
-      <c r="Q7" s="129"/>
-      <c r="R7" s="131"/>
+      <c r="Q7" s="128"/>
+      <c r="R7" s="130"/>
       <c r="T7" s="77"/>
     </row>
     <row r="8" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2516,10 +2518,10 @@
         <v>6.2</v>
       </c>
       <c r="P12" s="106"/>
-      <c r="Q12" s="128" t="s">
+      <c r="Q12" s="127" t="s">
         <v>90</v>
       </c>
-      <c r="R12" s="130"/>
+      <c r="R12" s="129"/>
       <c r="T12" s="77"/>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.35">
@@ -2569,8 +2571,8 @@
         <v>6.2</v>
       </c>
       <c r="P13" s="97"/>
-      <c r="Q13" s="129"/>
-      <c r="R13" s="131"/>
+      <c r="Q13" s="128"/>
+      <c r="R13" s="130"/>
       <c r="T13" s="77"/>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.35">
@@ -2620,8 +2622,8 @@
         <v>6.2</v>
       </c>
       <c r="P14" s="97"/>
-      <c r="Q14" s="129"/>
-      <c r="R14" s="131"/>
+      <c r="Q14" s="128"/>
+      <c r="R14" s="130"/>
       <c r="T14" s="77"/>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.35">
@@ -2671,8 +2673,8 @@
         <v>6.15</v>
       </c>
       <c r="P15" s="97"/>
-      <c r="Q15" s="129"/>
-      <c r="R15" s="131"/>
+      <c r="Q15" s="128"/>
+      <c r="R15" s="130"/>
       <c r="T15" s="77"/>
     </row>
     <row r="16" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2722,8 +2724,8 @@
         <v>6.15</v>
       </c>
       <c r="P16" s="97"/>
-      <c r="Q16" s="129"/>
-      <c r="R16" s="131"/>
+      <c r="Q16" s="128"/>
+      <c r="R16" s="130"/>
       <c r="T16" s="77"/>
     </row>
     <row r="17" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -2786,7 +2788,7 @@
     <col min="11" max="13" width="11.36328125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="8.1796875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="6.90625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.36328125" customWidth="1"/>
+    <col min="16" max="17" width="10.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
@@ -2836,6 +2838,9 @@
       <c r="P2" s="72" t="s">
         <v>64</v>
       </c>
+      <c r="Q2" s="72" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="3" spans="1:17" s="52" customFormat="1" ht="14.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="51"/>
@@ -2887,7 +2892,7 @@
         <f>N3*O3</f>
         <v>7618.7666666666664</v>
       </c>
-      <c r="Q3" s="77"/>
+      <c r="Q3" s="106"/>
     </row>
     <row r="4" spans="1:17" s="52" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="51"/>
@@ -2939,7 +2944,7 @@
         <f t="shared" ref="P4:P7" si="0">N4*O4</f>
         <v>1862.0666666666666</v>
       </c>
-      <c r="Q4" s="77"/>
+      <c r="Q4" s="106"/>
     </row>
     <row r="5" spans="1:17" s="52" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="51"/>
@@ -2991,7 +2996,7 @@
         <f t="shared" si="0"/>
         <v>6293</v>
       </c>
-      <c r="Q5" s="77"/>
+      <c r="Q5" s="106"/>
     </row>
     <row r="6" spans="1:17" s="52" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="51"/>
@@ -3043,7 +3048,7 @@
         <f t="shared" si="0"/>
         <v>6076</v>
       </c>
-      <c r="Q6" s="77"/>
+      <c r="Q6" s="106"/>
     </row>
     <row r="7" spans="1:17" s="52" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="51"/>
@@ -3095,7 +3100,7 @@
         <f t="shared" si="0"/>
         <v>3145.7250000000004</v>
       </c>
-      <c r="Q7" s="77"/>
+      <c r="Q7" s="106"/>
     </row>
     <row r="8" spans="1:17" s="52" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="51"/>
@@ -3124,6 +3129,7 @@
       <c r="P8" s="95" t="s">
         <v>73</v>
       </c>
+      <c r="Q8" s="95"/>
     </row>
     <row r="10" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="11" spans="1:17" s="52" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
@@ -3176,7 +3182,7 @@
         <f>N11*O11</f>
         <v>7618.7666666666664</v>
       </c>
-      <c r="Q11" s="77"/>
+      <c r="Q11" s="106"/>
     </row>
     <row r="12" spans="1:17" s="52" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="51"/>
@@ -3195,7 +3201,7 @@
       <c r="N12" s="123"/>
       <c r="O12" s="124"/>
       <c r="P12" s="125"/>
-      <c r="Q12" s="77"/>
+      <c r="Q12" s="125"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.35">
       <c r="O13" t="s">
@@ -3205,6 +3211,7 @@
         <f>P11</f>
         <v>7618.7666666666664</v>
       </c>
+      <c r="Q13" s="117"/>
     </row>
     <row r="14" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="15" spans="1:17" s="52" customFormat="1" x14ac:dyDescent="0.35">
@@ -3257,7 +3264,7 @@
         <f t="shared" ref="P15" si="1">N15*O15</f>
         <v>1862.0666666666666</v>
       </c>
-      <c r="Q15" s="77"/>
+      <c r="Q15" s="106"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.35">
       <c r="O16" t="s">
@@ -3267,6 +3274,7 @@
         <f>P15</f>
         <v>1862.0666666666666</v>
       </c>
+      <c r="Q16" s="117"/>
     </row>
     <row r="17" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="18" spans="1:17" s="52" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -3319,7 +3327,7 @@
         <f t="shared" ref="P18:P19" si="2">N18*O18</f>
         <v>6293</v>
       </c>
-      <c r="Q18" s="77"/>
+      <c r="Q18" s="106"/>
     </row>
     <row r="19" spans="1:17" s="52" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="51"/>
@@ -3343,7 +3351,7 @@
       </c>
       <c r="H19" s="75">
         <f>N19*6</f>
-        <v>1470</v>
+        <v>0</v>
       </c>
       <c r="I19" s="85">
         <v>43603750</v>
@@ -3362,7 +3370,7 @@
       </c>
       <c r="N19" s="86">
         <f>Q19*70</f>
-        <v>245</v>
+        <v>0</v>
       </c>
       <c r="O19" s="87">
         <f>_xlfn.XLOOKUP(E19,'Master data'!$B:$B,'Master data'!$H:$H)</f>
@@ -3370,24 +3378,23 @@
       </c>
       <c r="P19" s="106">
         <f t="shared" si="2"/>
-        <v>1519</v>
-      </c>
-      <c r="Q19" s="126">
-        <v>3.5</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q19" s="106"/>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="H20" s="127">
+      <c r="H20" s="126">
         <f>H18+H19</f>
-        <v>7560</v>
+        <v>6090</v>
       </c>
       <c r="O20" t="s">
         <v>122</v>
       </c>
       <c r="P20" s="117">
         <f>SUM(P18:P19)</f>
-        <v>7812</v>
-      </c>
+        <v>6293</v>
+      </c>
+      <c r="Q20" s="117"/>
     </row>
     <row r="21" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="22" spans="1:17" s="52" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -3412,7 +3419,7 @@
       </c>
       <c r="H22" s="75">
         <f>H6-H19</f>
-        <v>4410</v>
+        <v>5880</v>
       </c>
       <c r="I22" s="85">
         <v>43603750</v>
@@ -3431,7 +3438,7 @@
       </c>
       <c r="N22" s="86">
         <f>N6-N19</f>
-        <v>735</v>
+        <v>980</v>
       </c>
       <c r="O22" s="87">
         <f>_xlfn.XLOOKUP(E22,'Master data'!$B:$B,'Master data'!$H:$H)</f>
@@ -3439,9 +3446,9 @@
       </c>
       <c r="P22" s="106">
         <f t="shared" ref="P22:P23" si="3">N22*O22</f>
-        <v>4557</v>
-      </c>
-      <c r="Q22" s="77"/>
+        <v>6076</v>
+      </c>
+      <c r="Q22" s="106"/>
     </row>
     <row r="23" spans="1:17" s="52" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="51"/>
@@ -3493,20 +3500,21 @@
         <f t="shared" si="3"/>
         <v>3145.7250000000004</v>
       </c>
-      <c r="Q23" s="77"/>
+      <c r="Q23" s="106"/>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="H24" s="127">
+      <c r="H24" s="126">
         <f>H22+H23</f>
-        <v>10548</v>
+        <v>12018</v>
       </c>
       <c r="O24" t="s">
         <v>123</v>
       </c>
       <c r="P24" s="117">
         <f>P22+P23</f>
-        <v>7702.7250000000004</v>
-      </c>
+        <v>9221.7250000000004</v>
+      </c>
+      <c r="Q24" s="117"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5183,14 +5191,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2b71f93c-9935-46f3-83c7-0ee45f40cc46">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="fbbcc733-362e-45f8-a41b-1c2eddb78e13" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5401,21 +5407,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2b71f93c-9935-46f3-83c7-0ee45f40cc46">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="fbbcc733-362e-45f8-a41b-1c2eddb78e13" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48B4DA36-310A-48FF-A575-A75EDC20FDC5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9F6C60-CD63-4A80-821B-90406191FB43}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2b71f93c-9935-46f3-83c7-0ee45f40cc46"/>
-    <ds:schemaRef ds:uri="fbbcc733-362e-45f8-a41b-1c2eddb78e13"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5440,9 +5445,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9F6C60-CD63-4A80-821B-90406191FB43}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48B4DA36-310A-48FF-A575-A75EDC20FDC5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2b71f93c-9935-46f3-83c7-0ee45f40cc46"/>
+    <ds:schemaRef ds:uri="fbbcc733-362e-45f8-a41b-1c2eddb78e13"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>